<commit_message>
research: add Inferences sheet (positive/negative synthesis)
Executive synthesis of the home-loan review research as a new workbook tab:
positive inferences (demand validated, research-before-apply, support as
differentiator, DSA channel) and negative inferences (reliability kills good
products, cost/interest anger, after-sales black hole, trust/data, onboarding
friction, inflated ratings), plus a competitor-pain -> DhanIQ-answer mapping.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/ambak-competitor-reviews.xlsx
+++ b/research/ambak-competitor-reviews.xlsx
@@ -4,13 +4,15 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Theme Analysis" sheetId="2" r:id="rId2"/>
-    <sheet name="All Reviews" sheetId="3" r:id="rId3"/>
+    <sheet name="Inferences" sheetId="2" r:id="rId2"/>
+    <sheet name="Theme Analysis" sheetId="3" r:id="rId3"/>
+    <sheet name="All Reviews" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Summary'!A1:O8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Theme Analysis'!A1:K8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'All Reviews'!A1:G334</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Theme Analysis'!A1:K8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'All Reviews'!A1:G334</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -792,20 +794,247 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C29"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="52.83203125" customWidth="1"/>
+    <col min="3" max="3" width="95.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Ambak &amp; Home-Loan Competitor Reviews - Inferences</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Scope: home-loan reviews only (India Google Play + Apple App Store). See 'Theme Analysis' for method &amp; caveats.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Generated: 2026-09-13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>POSITIVE INFERENCES (what the market rewards)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>#</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Inference</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Evidence / basis</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>1</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Demand for honest home-loan comparison is proven</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Credit Dharma's home-loan users praise exactly DhanIQ's concept: 'find lowest home loan rates across banks', 'very accurate home-loan calculation', 'better than other EMI calculator apps'. Direct validation of the core idea.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Borrowers research months before they apply</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Paisabazaar home-loan reviews show a 'prepare first' audience checking credit score/report 6-7 months ahead of applying. A real top-of-funnel window for a no-pressure tool to earn trust early.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>3</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Good human support is a genuine differentiator</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Where it shows up it is loved: Ambak (JustDial 4.4, 'smooth process, supportive staff'), Paisabazaar ('seamless home-loan support/disbursal'). Service quality, not just rates, moves sentiment.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>4</v>
+      </c>
+      <c r="B10" t="str">
+        <v>The partner / agent (DSA) channel works</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Ambak Saathi (4.68) and OneAndro cross-sell mentions show the B2B2C distribution model has satisfied users on the supply side.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>NEGATIVE INFERENCES (recurring pain - avoid / exploit)</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>#</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Inference</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Evidence / basis</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>1</v>
+      </c>
+      <c r="B14" t="str">
+        <v>App reliability kills otherwise-great products</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Credit Dharma has the best concept but the LOWEST rating (3.79), dragged down by ~48 mentions of login failures / 'app won't open' / broken sign-up. The idea lands; execution leaks. Reliability beats features.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Interest rates &amp; hidden cost are a raw nerve</v>
+      </c>
+      <c r="C15" t="str">
+        <v>HomeFirst draws furious home-loan reviews: 'rate of interest bahut zyada', 'heavy ROI, avoid this'. Cost opacity generates real anger - precisely DhanIQ's 'true cost' wedge.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>3</v>
+      </c>
+      <c r="B16" t="str">
+        <v>After-sales service is a black hole</v>
+      </c>
+      <c r="C16" t="str">
+        <v>HomeFirst's loudest theme (~25 mentions) is unreachable customer care plus statement/payment disputes ('paid Rs.20,000, statement shows Rs.12,000'). Post-disbursal neglect destroys hard-won trust.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>4</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Trust erodes on bait-and-switch and data misuse</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Adjacent signal (Paisabazaar): 'pre-approved then rejected - felt cheated', 'selling my data'. Ambak markets 'no pushy calls' yet gets a persistent-calls complaint. Marketing that contradicts lived experience is punished.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>5</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Onboarding friction loses people</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Andromeda's negatives cluster on KYC / activation stuck for weeks. Slow verification is an early drop-off point.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>6</v>
+      </c>
+      <c r="B19" t="str">
+        <v>High star-ratings can be manufactured</v>
+      </c>
+      <c r="C19" t="str">
+        <v>GoCredit's near-perfect 4.75 is built on generic one-word 5-star text - reads as solicited. Don't benchmark against inflated ratings.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>IMPLICATIONS FOR DHANIQ</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Competitor pain</v>
+      </c>
+      <c r="B22" t="str">
+        <v>DhanIQ's answer</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Opaque / high cost, 'hidden' rates</v>
+      </c>
+      <c r="B23" t="str">
+        <v>True-cost / effective-APR computation</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Pushy calls, data selling</v>
+      </c>
+      <c r="B24" t="str">
+        <v>On-device; nothing leaves the device; no calls</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Bait 'pre-approved' then rejected</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Advice-neutral; no lead-gen; no recommendations</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>App won't open / login bugs</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Opportunity: win on reliability (Credit Dharma's weak spot)</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>BOTTOM LINE</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+      <c r="B29" t="str">
+        <v>Demand for the product is validated; market leaders lose on trust, transparency, and app reliability - the exact axes DhanIQ is built to win. Caution: a great concept dies on a broken first-run, so reliability and a frictionless first use matter as much as the finance engine.</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A20:C20"/>
+  </mergeCells>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K17"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="70.83203125" customWidth="1"/>
-    <col min="10" max="10" width="55.83203125" customWidth="1"/>
-    <col min="11" max="11" width="45.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1156,7 +1385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G334"/>
   <sheetData>

</xml_diff>